<commit_message>
stable version of ddt and ddt perform in registration page
</commit_message>
<xml_diff>
--- a/TestData/registration_data.xlsx
+++ b/TestData/registration_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashish_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C0E4F6-FD42-45FB-AD19-B33D033543AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4574C1F9-9030-4C6F-B5EF-32533CB38258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AD059314-005E-446C-AE50-52F4E115D9E8}"/>
   </bookViews>
@@ -34,13 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
-  <si>
-    <t>username</t>
-  </si>
-  <si>
-    <t>email_address</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
   <si>
     <t>password</t>
   </si>
@@ -87,24 +81,12 @@
     <t>mobile_number</t>
   </si>
   <si>
-    <t>ashish</t>
-  </si>
-  <si>
-    <t>sa635am@outlook.com</t>
-  </si>
-  <si>
     <t>saran@002</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>April</t>
   </si>
   <si>
-    <t>1994</t>
-  </si>
-  <si>
     <t>dube</t>
   </si>
   <si>
@@ -129,47 +111,65 @@
     <t>Yavatmal</t>
   </si>
   <si>
-    <t>445563</t>
-  </si>
-  <si>
-    <t>9988774455</t>
-  </si>
-  <si>
     <t>expected_result</t>
   </si>
   <si>
-    <t>pass</t>
-  </si>
-  <si>
-    <t>ashishkho</t>
-  </si>
-  <si>
-    <t>sant@gmail.com</t>
-  </si>
-  <si>
-    <t>fail</t>
-  </si>
-  <si>
     <t>signup_username</t>
   </si>
   <si>
-    <t>signup_email</t>
-  </si>
-  <si>
-    <t>sahar mahune</t>
-  </si>
-  <si>
-    <t>sagar@outlook.com</t>
-  </si>
-  <si>
     <t>sahar</t>
+  </si>
+  <si>
+    <t>signup_email_address</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>abdul</t>
+  </si>
+  <si>
+    <t>sahil</t>
+  </si>
+  <si>
+    <t>sahu@78</t>
+  </si>
+  <si>
+    <t>shaikh</t>
+  </si>
+  <si>
+    <t>tata</t>
+  </si>
+  <si>
+    <t>pune</t>
+  </si>
+  <si>
+    <t>chichwad</t>
+  </si>
+  <si>
+    <t>hinjawadi</t>
+  </si>
+  <si>
+    <t>panjab</t>
+  </si>
+  <si>
+    <t>luhiyana</t>
+  </si>
+  <si>
+    <t>june25d@outlook.com</t>
+  </si>
+  <si>
+    <t>afs25al@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,6 +206,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -228,7 +234,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -236,6 +242,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -551,54 +564,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E30579E4-906A-4028-9E6D-19D6C2F3A8BA}">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="21.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="3"/>
+    <col min="7" max="7" width="14.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>6</v>
@@ -627,126 +639,159 @@
       <c r="Q1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="D2" s="6">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="F2">
+        <v>1994</v>
+      </c>
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2">
+        <v>445563</v>
+      </c>
+      <c r="Q2">
+        <v>9988774455</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="D3" s="9">
+        <v>12</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="8">
+        <v>1985</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" t="s">
         <v>22</v>
       </c>
-      <c r="G2" t="s">
+      <c r="N3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q2" t="s">
+      <c r="P3" s="3">
+        <v>448552</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>8575</v>
+      </c>
+      <c r="R3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="R2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S2" t="s">
-        <v>32</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
@@ -764,9 +809,10 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{16DC758B-1D5C-4A7E-8842-6F3BC5E8E3F9}"/>
-    <hyperlink ref="H2" r:id="rId2" xr:uid="{D7109D52-FFFC-4129-9C80-2BA88BE733BF}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{5A841AD9-E1FF-4CA2-B628-528A5118FD5F}"/>
+    <hyperlink ref="B2" r:id="rId3" xr:uid="{0E9A779D-D128-4508-8EEF-377841F64607}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
stable version of ddt
</commit_message>
<xml_diff>
--- a/TestData/registration_data.xlsx
+++ b/TestData/registration_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashish_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4574C1F9-9030-4C6F-B5EF-32533CB38258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2330CECD-6EC6-4B78-8522-C8E2C063C48E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AD059314-005E-446C-AE50-52F4E115D9E8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>password</t>
   </si>
@@ -81,9 +81,6 @@
     <t>mobile_number</t>
   </si>
   <si>
-    <t>saran@002</t>
-  </si>
-  <si>
     <t>April</t>
   </si>
   <si>
@@ -163,6 +160,12 @@
   </si>
   <si>
     <t>afs25al@gmail.com</t>
+  </si>
+  <si>
+    <t>failure</t>
+  </si>
+  <si>
+    <t>Ash@654</t>
   </si>
 </sst>
 </file>
@@ -589,10 +592,10 @@
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -640,54 +643,54 @@
         <v>14</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
+        <v>40</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="D2" s="6">
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F2">
         <v>1994</v>
       </c>
       <c r="G2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>18</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>20</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>21</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>22</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>23</v>
-      </c>
-      <c r="O2" t="s">
-        <v>24</v>
       </c>
       <c r="P2">
         <v>445563</v>
@@ -696,63 +699,60 @@
         <v>9988774455</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="D3" s="9">
         <v>12</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F3" s="8">
         <v>1985</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="M3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="P3" s="3">
         <v>448552</v>
       </c>
-      <c r="Q3" s="3">
-        <v>8575</v>
-      </c>
       <c r="R3" s="3" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
@@ -811,8 +811,9 @@
     <hyperlink ref="B3" r:id="rId1" xr:uid="{16DC758B-1D5C-4A7E-8842-6F3BC5E8E3F9}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{5A841AD9-E1FF-4CA2-B628-528A5118FD5F}"/>
     <hyperlink ref="B2" r:id="rId3" xr:uid="{0E9A779D-D128-4508-8EEF-377841F64607}"/>
+    <hyperlink ref="C2" r:id="rId4" xr:uid="{20D2E684-014D-4D73-B908-990C050ACC24}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
database connection and validate new reg records found in database
</commit_message>
<xml_diff>
--- a/TestData/registration_data.xlsx
+++ b/TestData/registration_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashish_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2330CECD-6EC6-4B78-8522-C8E2C063C48E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{401B2443-0344-48A7-BE1E-C99258B01CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AD059314-005E-446C-AE50-52F4E115D9E8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
   <si>
     <t>password</t>
   </si>
@@ -87,27 +87,12 @@
     <t>dube</t>
   </si>
   <si>
-    <t>Mumbai</t>
-  </si>
-  <si>
-    <t>panchashl bagar</t>
-  </si>
-  <si>
-    <t>sane gurugi</t>
-  </si>
-  <si>
-    <t>bhag 2</t>
-  </si>
-  <si>
     <t>India</t>
   </si>
   <si>
     <t>Maharashtra</t>
   </si>
   <si>
-    <t>Yavatmal</t>
-  </si>
-  <si>
     <t>expected_result</t>
   </si>
   <si>
@@ -166,6 +151,45 @@
   </si>
   <si>
     <t>Ash@654</t>
+  </si>
+  <si>
+    <t>cognizant</t>
+  </si>
+  <si>
+    <t>vima nagar</t>
+  </si>
+  <si>
+    <t>chakan road</t>
+  </si>
+  <si>
+    <t>sen</t>
+  </si>
+  <si>
+    <t>HCL</t>
+  </si>
+  <si>
+    <t>ching pokali</t>
+  </si>
+  <si>
+    <t>muharji nagar</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Mihir</t>
+  </si>
+  <si>
+    <t>ac</t>
+  </si>
+  <si>
+    <t>asd@gmail.com</t>
+  </si>
+  <si>
+    <t>sd@256</t>
+  </si>
+  <si>
+    <t>March</t>
   </si>
 </sst>
 </file>
@@ -573,9 +597,9 @@
     <col min="1" max="1" width="24" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13" style="3" bestFit="1" customWidth="1"/>
@@ -592,10 +616,10 @@
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -643,18 +667,18 @@
         <v>14</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D2" s="6">
         <v>6</v>
@@ -666,97 +690,150 @@
         <v>1994</v>
       </c>
       <c r="G2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
         <v>16</v>
       </c>
       <c r="I2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" t="s">
         <v>17</v>
       </c>
-      <c r="J2" t="s">
+      <c r="N2" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L2" t="s">
-        <v>20</v>
-      </c>
-      <c r="M2" t="s">
-        <v>21</v>
-      </c>
-      <c r="N2" t="s">
-        <v>22</v>
-      </c>
       <c r="O2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="P2">
-        <v>445563</v>
+        <v>445566</v>
       </c>
       <c r="Q2">
-        <v>9988774455</v>
+        <v>7563225545</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D3" s="9">
         <v>12</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F3" s="8">
         <v>1985</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="L3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M3" t="s">
-        <v>21</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>39</v>
       </c>
       <c r="P3" s="3">
         <v>448552</v>
       </c>
       <c r="R3" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="7">
+        <v>25</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1996</v>
+      </c>
+      <c r="G4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A4"/>
+      <c r="I4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K4" t="s">
+        <v>45</v>
+      </c>
+      <c r="L4" t="s">
+        <v>46</v>
+      </c>
+      <c r="M4" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" t="s">
+        <v>46</v>
+      </c>
+      <c r="O4" t="s">
+        <v>46</v>
+      </c>
+      <c r="P4">
+        <v>123456</v>
+      </c>
+      <c r="Q4">
+        <v>9685632545</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5"/>
@@ -812,8 +889,10 @@
     <hyperlink ref="C3" r:id="rId2" xr:uid="{5A841AD9-E1FF-4CA2-B628-528A5118FD5F}"/>
     <hyperlink ref="B2" r:id="rId3" xr:uid="{0E9A779D-D128-4508-8EEF-377841F64607}"/>
     <hyperlink ref="C2" r:id="rId4" xr:uid="{20D2E684-014D-4D73-B908-990C050ACC24}"/>
+    <hyperlink ref="B4" r:id="rId5" xr:uid="{E25C19AE-6F8A-4E06-9CD5-09AFA394F5DE}"/>
+    <hyperlink ref="C4" r:id="rId6" xr:uid="{892040D2-7222-463D-9316-57A732A0E1DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
stable version of DataBase validation
</commit_message>
<xml_diff>
--- a/TestData/registration_data.xlsx
+++ b/TestData/registration_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashish_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{401B2443-0344-48A7-BE1E-C99258B01CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2755B7-3D11-41EA-B1E0-5ACA5CAD8CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AD059314-005E-446C-AE50-52F4E115D9E8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="41">
   <si>
     <t>password</t>
   </si>
@@ -147,9 +147,6 @@
     <t>afs25al@gmail.com</t>
   </si>
   <si>
-    <t>failure</t>
-  </si>
-  <si>
     <t>Ash@654</t>
   </si>
   <si>
@@ -160,36 +157,6 @@
   </si>
   <si>
     <t>chakan road</t>
-  </si>
-  <si>
-    <t>sen</t>
-  </si>
-  <si>
-    <t>HCL</t>
-  </si>
-  <si>
-    <t>ching pokali</t>
-  </si>
-  <si>
-    <t>muharji nagar</t>
-  </si>
-  <si>
-    <t>Delhi</t>
-  </si>
-  <si>
-    <t>Mihir</t>
-  </si>
-  <si>
-    <t>ac</t>
-  </si>
-  <si>
-    <t>asd@gmail.com</t>
-  </si>
-  <si>
-    <t>sd@256</t>
-  </si>
-  <si>
-    <t>March</t>
   </si>
 </sst>
 </file>
@@ -678,7 +645,7 @@
         <v>35</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2" s="6">
         <v>6</v>
@@ -696,13 +663,13 @@
         <v>16</v>
       </c>
       <c r="I2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J2" t="s">
         <v>39</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>40</v>
-      </c>
-      <c r="K2" t="s">
-        <v>41</v>
       </c>
       <c r="L2" t="s">
         <v>30</v>
@@ -775,65 +742,28 @@
       <c r="P3" s="3">
         <v>448552</v>
       </c>
+      <c r="Q3" s="3">
+        <v>9966778899</v>
+      </c>
       <c r="R3" s="3" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="7">
-        <v>25</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1996</v>
-      </c>
-      <c r="G4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" t="s">
-        <v>42</v>
-      </c>
-      <c r="I4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L4" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" t="s">
-        <v>46</v>
-      </c>
-      <c r="O4" t="s">
-        <v>46</v>
-      </c>
-      <c r="P4">
-        <v>123456</v>
-      </c>
-      <c r="Q4">
-        <v>9685632545</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>24</v>
-      </c>
+      <c r="A4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4"/>
+      <c r="N4"/>
+      <c r="O4"/>
+      <c r="P4"/>
+      <c r="Q4"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5"/>
@@ -889,10 +819,8 @@
     <hyperlink ref="C3" r:id="rId2" xr:uid="{5A841AD9-E1FF-4CA2-B628-528A5118FD5F}"/>
     <hyperlink ref="B2" r:id="rId3" xr:uid="{0E9A779D-D128-4508-8EEF-377841F64607}"/>
     <hyperlink ref="C2" r:id="rId4" xr:uid="{20D2E684-014D-4D73-B908-990C050ACC24}"/>
-    <hyperlink ref="B4" r:id="rId5" xr:uid="{E25C19AE-6F8A-4E06-9CD5-09AFA394F5DE}"/>
-    <hyperlink ref="C4" r:id="rId6" xr:uid="{892040D2-7222-463D-9316-57A732A0E1DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>